<commit_message>
fix(api): atomic counter increments, IP spoofing, and validation gaps
- Replace read-then-upsert counter logic with a compare-and-swap
  helper to prevent lost increments under concurrent requests
- Drop spoofable X-Forwarded-For fallback in rate limiter, trust
  only CF-Connecting-IP
- Add periodic cleanup of expired entries in the in-memory rate
  limit Map to prevent unbounded growth
- Apply existing query validation schema to /api/ai for consistency
  with /api/tools and /api/games
</commit_message>
<xml_diff>
--- a/tests/appium/reports/appium-report.xlsx
+++ b/tests/appium/reports/appium-report.xlsx
@@ -494,7 +494,7 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -543,7 +543,7 @@
         <v>15</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" t="s">
         <v>16</v>

</xml_diff>